<commit_message>
Work 11 March v1
</commit_message>
<xml_diff>
--- a/ICSummary/20250211/PerformanceSummaryJan2025.xlsx
+++ b/ICSummary/20250211/PerformanceSummaryJan2025.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/fa1b30dd86628461/FILE Backup/Kev/PYTHON Projects/AtchisonAnalyticsWebsite/ICSummary/20250211/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="372" documentId="8_{8585333A-8958-49B5-87CD-D3974D5B51CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DDB54A74-E467-4DAE-95F0-D1F79D3AE79E}"/>
+  <xr:revisionPtr revIDLastSave="373" documentId="8_{8585333A-8958-49B5-87CD-D3974D5B51CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{81C61DDD-705B-48FE-9BCE-E56880E9BDA2}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" firstSheet="1" activeTab="1" xr2:uid="{E02CCEAF-9CFD-4D4D-B2FA-7B81BC99F0F0}"/>
   </bookViews>
@@ -557,7 +557,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="65">
+  <cellXfs count="60">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -662,71 +662,64 @@
     <xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="2" fontId="4" fillId="5" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="4" fillId="5" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="4" fillId="5" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="4" fillId="5" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="2" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="2" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="3" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="3" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="4" fillId="5" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="4" fillId="5" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="4" fillId="5" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="2" fontId="4" fillId="5" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="2" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="7" fillId="2" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="7" fillId="2" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="3" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="3" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1087,15 +1080,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:12" s="25" customFormat="1" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B1" s="40" t="s">
+      <c r="B1" s="59" t="s">
         <v>24</v>
       </c>
-      <c r="C1" s="40"/>
-      <c r="D1" s="40"/>
-      <c r="E1" s="40"/>
-      <c r="F1" s="40"/>
-      <c r="G1" s="40"/>
-      <c r="H1" s="40"/>
+      <c r="C1" s="59"/>
+      <c r="D1" s="59"/>
+      <c r="E1" s="59"/>
+      <c r="F1" s="59"/>
+      <c r="G1" s="59"/>
+      <c r="H1" s="59"/>
       <c r="J1" s="32"/>
     </row>
     <row r="4" spans="2:12" s="25" customFormat="1" ht="42" customHeight="1" x14ac:dyDescent="0.25">
@@ -1790,64 +1783,63 @@
     <col min="10" max="10" width="3.42578125" customWidth="1"/>
     <col min="11" max="12" width="18.7109375" customWidth="1"/>
     <col min="13" max="13" width="3.42578125" customWidth="1"/>
-    <col min="14" max="14" width="18.7109375" style="46" customWidth="1"/>
-    <col min="15" max="15" width="18.7109375" customWidth="1"/>
+    <col min="14" max="15" width="18.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="2:15" s="25" customFormat="1" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B1" s="40" t="s">
+      <c r="B1" s="59" t="s">
         <v>25</v>
       </c>
-      <c r="C1" s="40"/>
-      <c r="D1" s="40"/>
-      <c r="E1" s="40"/>
-      <c r="F1" s="40"/>
-      <c r="G1" s="40"/>
-      <c r="H1" s="40"/>
+      <c r="C1" s="59"/>
+      <c r="D1" s="59"/>
+      <c r="E1" s="59"/>
+      <c r="F1" s="59"/>
+      <c r="G1" s="59"/>
+      <c r="H1" s="59"/>
       <c r="I1" s="39"/>
       <c r="K1" s="32"/>
-      <c r="N1" s="45"/>
+      <c r="N1" s="32"/>
     </row>
     <row r="4" spans="2:15" s="25" customFormat="1" ht="42" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B4" s="52" t="s">
+      <c r="B4" s="46" t="s">
         <v>10</v>
       </c>
-      <c r="C4" s="59" t="s">
+      <c r="C4" s="53" t="s">
         <v>0</v>
       </c>
-      <c r="D4" s="55" t="s">
+      <c r="D4" s="49" t="s">
         <v>1</v>
       </c>
-      <c r="E4" s="55" t="s">
+      <c r="E4" s="49" t="s">
         <v>2</v>
       </c>
-      <c r="F4" s="55" t="s">
+      <c r="F4" s="49" t="s">
         <v>3</v>
       </c>
-      <c r="G4" s="55" t="s">
+      <c r="G4" s="49" t="s">
         <v>4</v>
       </c>
-      <c r="H4" s="55" t="s">
+      <c r="H4" s="49" t="s">
         <v>23</v>
       </c>
-      <c r="I4" s="56" t="s">
+      <c r="I4" s="50" t="s">
         <v>26</v>
       </c>
-      <c r="K4" s="61" t="s">
+      <c r="K4" s="55" t="s">
         <v>29</v>
       </c>
-      <c r="L4" s="62" t="s">
+      <c r="L4" s="56" t="s">
         <v>28</v>
       </c>
-      <c r="N4" s="61" t="s">
+      <c r="N4" s="55" t="s">
         <v>30</v>
       </c>
-      <c r="O4" s="62" t="s">
+      <c r="O4" s="56" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="5" spans="2:15" s="1" customFormat="1" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="B5" s="57" t="s">
+      <c r="B5" s="51" t="s">
         <v>6</v>
       </c>
       <c r="C5" s="3">
@@ -1872,22 +1864,22 @@
         <v>11.73</v>
       </c>
       <c r="J5" s="6"/>
-      <c r="K5" s="42">
+      <c r="K5" s="41">
         <v>7.61</v>
       </c>
-      <c r="L5" s="41">
+      <c r="L5" s="40">
         <v>1.1599999999999999</v>
       </c>
       <c r="M5" s="6"/>
-      <c r="N5" s="42">
+      <c r="N5" s="41">
         <v>6.57</v>
       </c>
-      <c r="O5" s="41">
+      <c r="O5" s="40">
         <v>-7.27</v>
       </c>
     </row>
     <row r="6" spans="2:15" s="1" customFormat="1" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="B6" s="57" t="s">
+      <c r="B6" s="51" t="s">
         <v>7</v>
       </c>
       <c r="C6" s="8">
@@ -1912,22 +1904,22 @@
         <v>11.57</v>
       </c>
       <c r="J6" s="6"/>
-      <c r="K6" s="47">
+      <c r="K6" s="43">
         <v>6.68</v>
       </c>
-      <c r="L6" s="43">
+      <c r="L6" s="42">
         <v>0.9</v>
       </c>
       <c r="M6" s="6"/>
-      <c r="N6" s="47">
+      <c r="N6" s="43">
         <v>7.4</v>
       </c>
-      <c r="O6" s="43">
+      <c r="O6" s="42">
         <v>-8.7100000000000009</v>
       </c>
     </row>
     <row r="7" spans="2:15" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B7" s="60" t="s">
+      <c r="B7" s="54" t="s">
         <v>9</v>
       </c>
       <c r="C7" s="10">
@@ -1952,7 +1944,7 @@
         <v>9.56</v>
       </c>
       <c r="J7" s="13"/>
-      <c r="K7" s="63">
+      <c r="K7" s="57">
         <v>4.9800000000000004</v>
       </c>
       <c r="L7" s="12">
@@ -1967,7 +1959,7 @@
       </c>
     </row>
     <row r="8" spans="2:15" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B8" s="58" t="s">
+      <c r="B8" s="52" t="s">
         <v>12</v>
       </c>
       <c r="C8" s="14"/>
@@ -1983,10 +1975,9 @@
       <c r="I8" s="16">
         <v>3.38</v>
       </c>
-      <c r="K8" s="64">
+      <c r="K8" s="58">
         <v>4.58</v>
       </c>
-      <c r="N8" s="48"/>
     </row>
     <row r="9" spans="2:15" x14ac:dyDescent="0.25">
       <c r="C9" s="17"/>
@@ -1997,10 +1988,10 @@
       <c r="H9" s="17"/>
       <c r="I9" s="17"/>
       <c r="J9" s="17"/>
-      <c r="K9" s="44"/>
+      <c r="K9" s="17"/>
       <c r="L9" s="17"/>
       <c r="M9" s="17"/>
-      <c r="N9" s="44"/>
+      <c r="N9" s="17"/>
       <c r="O9" s="17"/>
     </row>
     <row r="10" spans="2:15" s="1" customFormat="1" ht="18.75" x14ac:dyDescent="0.25">
@@ -2029,17 +2020,17 @@
         <v>13.65</v>
       </c>
       <c r="J10" s="6"/>
-      <c r="K10" s="42">
+      <c r="K10" s="41">
         <v>8.92</v>
       </c>
-      <c r="L10" s="41">
+      <c r="L10" s="40">
         <v>1.1399999999999999</v>
       </c>
       <c r="M10" s="6"/>
-      <c r="N10" s="42">
+      <c r="N10" s="41">
         <v>7.81</v>
       </c>
-      <c r="O10" s="41">
+      <c r="O10" s="40">
         <v>-8.4700000000000006</v>
       </c>
     </row>
@@ -2069,17 +2060,17 @@
         <v>13.58</v>
       </c>
       <c r="J11" s="6"/>
-      <c r="K11" s="47">
+      <c r="K11" s="43">
         <v>8.15</v>
       </c>
-      <c r="L11" s="43">
+      <c r="L11" s="42">
         <v>0.95</v>
       </c>
       <c r="M11" s="6"/>
-      <c r="N11" s="47">
+      <c r="N11" s="43">
         <v>8.58</v>
       </c>
-      <c r="O11" s="43">
+      <c r="O11" s="42">
         <v>-9.82</v>
       </c>
     </row>
@@ -2109,7 +2100,7 @@
         <v>11.8</v>
       </c>
       <c r="J12" s="17"/>
-      <c r="K12" s="63">
+      <c r="K12" s="57">
         <v>6.3</v>
       </c>
       <c r="L12" s="12">
@@ -2144,12 +2135,12 @@
         <v>3.38</v>
       </c>
       <c r="J13" s="13"/>
-      <c r="K13" s="64">
+      <c r="K13" s="58">
         <f>K8</f>
         <v>4.58</v>
       </c>
       <c r="M13" s="13"/>
-      <c r="N13" s="49"/>
+      <c r="N13" s="13"/>
     </row>
     <row r="14" spans="2:15" x14ac:dyDescent="0.25">
       <c r="C14" s="17"/>
@@ -2160,10 +2151,10 @@
       <c r="H14" s="17"/>
       <c r="I14" s="17"/>
       <c r="J14" s="17"/>
-      <c r="K14" s="44"/>
+      <c r="K14" s="17"/>
       <c r="L14" s="17"/>
       <c r="M14" s="17"/>
-      <c r="N14" s="44"/>
+      <c r="N14" s="17"/>
       <c r="O14" s="17"/>
     </row>
     <row r="15" spans="2:15" x14ac:dyDescent="0.25">
@@ -2175,10 +2166,10 @@
       <c r="H15" s="17"/>
       <c r="I15" s="17"/>
       <c r="J15" s="17"/>
-      <c r="K15" s="44"/>
+      <c r="K15" s="17"/>
       <c r="L15" s="17"/>
       <c r="M15" s="17"/>
-      <c r="N15" s="44"/>
+      <c r="N15" s="17"/>
       <c r="O15" s="17"/>
     </row>
     <row r="16" spans="2:15" x14ac:dyDescent="0.25">
@@ -2190,54 +2181,54 @@
       <c r="H16" s="17"/>
       <c r="I16" s="17"/>
       <c r="J16" s="17"/>
-      <c r="K16" s="44"/>
+      <c r="K16" s="17"/>
       <c r="L16" s="17"/>
       <c r="M16" s="17"/>
-      <c r="N16" s="44"/>
+      <c r="N16" s="17"/>
       <c r="O16" s="17"/>
     </row>
     <row r="17" spans="2:15" s="25" customFormat="1" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B17" s="52" t="s">
+      <c r="B17" s="46" t="s">
         <v>11</v>
       </c>
-      <c r="C17" s="53" t="s">
+      <c r="C17" s="47" t="s">
         <v>0</v>
       </c>
-      <c r="D17" s="54" t="s">
+      <c r="D17" s="48" t="s">
         <v>1</v>
       </c>
-      <c r="E17" s="54" t="s">
+      <c r="E17" s="48" t="s">
         <v>2</v>
       </c>
-      <c r="F17" s="54" t="s">
+      <c r="F17" s="48" t="s">
         <v>3</v>
       </c>
-      <c r="G17" s="54" t="s">
+      <c r="G17" s="48" t="s">
         <v>4</v>
       </c>
-      <c r="H17" s="55" t="s">
+      <c r="H17" s="49" t="s">
         <v>23</v>
       </c>
-      <c r="I17" s="56" t="s">
+      <c r="I17" s="50" t="s">
         <v>26</v>
       </c>
       <c r="J17" s="28"/>
-      <c r="K17" s="50" t="s">
+      <c r="K17" s="44" t="s">
         <v>19</v>
       </c>
-      <c r="L17" s="51" t="s">
+      <c r="L17" s="45" t="s">
         <v>28</v>
       </c>
       <c r="M17" s="28"/>
-      <c r="N17" s="50" t="s">
+      <c r="N17" s="44" t="s">
         <v>30</v>
       </c>
-      <c r="O17" s="51" t="s">
+      <c r="O17" s="45" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="18" spans="2:15" s="1" customFormat="1" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="B18" s="57" t="s">
+      <c r="B18" s="51" t="s">
         <v>15</v>
       </c>
       <c r="C18" s="3">
@@ -2262,22 +2253,22 @@
         <v>13.5</v>
       </c>
       <c r="J18" s="6"/>
-      <c r="K18" s="47">
+      <c r="K18" s="43">
         <v>11.25</v>
       </c>
-      <c r="L18" s="43">
+      <c r="L18" s="42">
         <v>0.86</v>
       </c>
       <c r="M18" s="6"/>
-      <c r="N18" s="47">
+      <c r="N18" s="43">
         <v>13.03</v>
       </c>
-      <c r="O18" s="43">
+      <c r="O18" s="42">
         <v>-12.52</v>
       </c>
     </row>
     <row r="19" spans="2:15" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B19" s="58" t="s">
+      <c r="B19" s="52" t="s">
         <v>9</v>
       </c>
       <c r="C19" s="14">
@@ -2319,17 +2310,17 @@
     <row r="20" spans="2:15" x14ac:dyDescent="0.25">
       <c r="C20" s="17"/>
       <c r="D20" s="17"/>
-      <c r="E20" s="44"/>
-      <c r="F20" s="44"/>
-      <c r="G20" s="44"/>
-      <c r="H20" s="44"/>
-      <c r="I20" s="44"/>
+      <c r="E20" s="17"/>
+      <c r="F20" s="17"/>
+      <c r="G20" s="17"/>
+      <c r="H20" s="17"/>
+      <c r="I20" s="17"/>
       <c r="J20" s="17"/>
-      <c r="K20" s="44"/>
-      <c r="L20" s="44"/>
+      <c r="K20" s="17"/>
+      <c r="L20" s="17"/>
       <c r="M20" s="17"/>
-      <c r="N20" s="44"/>
-      <c r="O20" s="44"/>
+      <c r="N20" s="17"/>
+      <c r="O20" s="17"/>
     </row>
     <row r="21" spans="2:15" ht="18.75" x14ac:dyDescent="0.25">
       <c r="B21" s="29" t="s">
@@ -2357,17 +2348,17 @@
         <v>24.25</v>
       </c>
       <c r="J21" s="17"/>
-      <c r="K21" s="47">
+      <c r="K21" s="43">
         <v>12.61</v>
       </c>
-      <c r="L21" s="43">
+      <c r="L21" s="42">
         <v>1.1399999999999999</v>
       </c>
       <c r="M21" s="17"/>
-      <c r="N21" s="42">
+      <c r="N21" s="41">
         <v>11.11</v>
       </c>
-      <c r="O21" s="43">
+      <c r="O21" s="42">
         <v>-10.79</v>
       </c>
     </row>
@@ -2414,17 +2405,17 @@
     <row r="23" spans="2:15" x14ac:dyDescent="0.25">
       <c r="C23" s="17"/>
       <c r="D23" s="17"/>
-      <c r="E23" s="44"/>
-      <c r="F23" s="44"/>
-      <c r="G23" s="44"/>
-      <c r="H23" s="44"/>
-      <c r="I23" s="44"/>
+      <c r="E23" s="17"/>
+      <c r="F23" s="17"/>
+      <c r="G23" s="17"/>
+      <c r="H23" s="17"/>
+      <c r="I23" s="17"/>
       <c r="J23" s="17"/>
-      <c r="K23" s="44"/>
-      <c r="L23" s="44"/>
+      <c r="K23" s="17"/>
+      <c r="L23" s="17"/>
       <c r="M23" s="17"/>
-      <c r="N23" s="44"/>
-      <c r="O23" s="44"/>
+      <c r="N23" s="17"/>
+      <c r="O23" s="17"/>
     </row>
     <row r="24" spans="2:15" ht="18.75" x14ac:dyDescent="0.25">
       <c r="B24" s="29" t="s">
@@ -2452,17 +2443,17 @@
         <v>7.29</v>
       </c>
       <c r="J24" s="17"/>
-      <c r="K24" s="47">
+      <c r="K24" s="43">
         <v>2.08</v>
       </c>
-      <c r="L24" s="43">
+      <c r="L24" s="42">
         <v>0.16</v>
       </c>
       <c r="M24" s="17"/>
-      <c r="N24" s="42">
+      <c r="N24" s="41">
         <v>12.91</v>
       </c>
-      <c r="O24" s="43">
+      <c r="O24" s="42">
         <v>-16.190000000000001</v>
       </c>
     </row>
@@ -2509,17 +2500,17 @@
     <row r="26" spans="2:15" x14ac:dyDescent="0.25">
       <c r="C26" s="17"/>
       <c r="D26" s="17"/>
-      <c r="E26" s="44"/>
-      <c r="F26" s="44"/>
-      <c r="G26" s="44"/>
-      <c r="H26" s="44"/>
-      <c r="I26" s="44"/>
+      <c r="E26" s="17"/>
+      <c r="F26" s="17"/>
+      <c r="G26" s="17"/>
+      <c r="H26" s="17"/>
+      <c r="I26" s="17"/>
       <c r="J26" s="17"/>
-      <c r="K26" s="44"/>
-      <c r="L26" s="44"/>
+      <c r="K26" s="17"/>
+      <c r="L26" s="17"/>
       <c r="M26" s="17"/>
-      <c r="N26" s="44"/>
-      <c r="O26" s="44"/>
+      <c r="N26" s="17"/>
+      <c r="O26" s="17"/>
     </row>
     <row r="27" spans="2:15" ht="18.75" x14ac:dyDescent="0.25">
       <c r="B27" s="29" t="s">
@@ -2547,17 +2538,17 @@
         <v>8.7100000000000009</v>
       </c>
       <c r="J27" s="17"/>
-      <c r="K27" s="47">
+      <c r="K27" s="43">
         <v>6.21</v>
       </c>
-      <c r="L27" s="43">
+      <c r="L27" s="42">
         <v>1.6</v>
       </c>
       <c r="M27" s="17"/>
-      <c r="N27" s="42">
+      <c r="N27" s="41">
         <v>3.89</v>
       </c>
-      <c r="O27" s="43">
+      <c r="O27" s="42">
         <v>-3.31</v>
       </c>
     </row>
@@ -2604,17 +2595,17 @@
     <row r="29" spans="2:15" x14ac:dyDescent="0.25">
       <c r="C29" s="17"/>
       <c r="D29" s="17"/>
-      <c r="E29" s="44"/>
-      <c r="F29" s="44"/>
-      <c r="G29" s="44"/>
-      <c r="H29" s="44"/>
-      <c r="I29" s="44"/>
+      <c r="E29" s="17"/>
+      <c r="F29" s="17"/>
+      <c r="G29" s="17"/>
+      <c r="H29" s="17"/>
+      <c r="I29" s="17"/>
       <c r="J29" s="17"/>
-      <c r="K29" s="44"/>
-      <c r="L29" s="44"/>
+      <c r="K29" s="17"/>
+      <c r="L29" s="17"/>
       <c r="M29" s="17"/>
-      <c r="N29" s="44"/>
-      <c r="O29" s="44"/>
+      <c r="N29" s="17"/>
+      <c r="O29" s="17"/>
     </row>
     <row r="30" spans="2:15" ht="18.75" x14ac:dyDescent="0.25">
       <c r="B30" s="29" t="s">
@@ -2642,17 +2633,17 @@
         <v>3.78</v>
       </c>
       <c r="J30" s="17"/>
-      <c r="K30" s="47">
+      <c r="K30" s="43">
         <v>-0.7</v>
       </c>
-      <c r="L30" s="43">
+      <c r="L30" s="42">
         <v>-0.11</v>
       </c>
       <c r="M30" s="17"/>
-      <c r="N30" s="42">
+      <c r="N30" s="41">
         <v>6.35</v>
       </c>
-      <c r="O30" s="43">
+      <c r="O30" s="42">
         <v>-10.23</v>
       </c>
     </row>
@@ -2699,17 +2690,17 @@
     <row r="32" spans="2:15" x14ac:dyDescent="0.25">
       <c r="C32" s="17"/>
       <c r="D32" s="17"/>
-      <c r="E32" s="44"/>
-      <c r="F32" s="44"/>
-      <c r="G32" s="44"/>
-      <c r="H32" s="44"/>
-      <c r="I32" s="44"/>
+      <c r="E32" s="17"/>
+      <c r="F32" s="17"/>
+      <c r="G32" s="17"/>
+      <c r="H32" s="17"/>
+      <c r="I32" s="17"/>
       <c r="J32" s="17"/>
-      <c r="K32" s="44"/>
-      <c r="L32" s="44"/>
+      <c r="K32" s="17"/>
+      <c r="L32" s="17"/>
       <c r="M32" s="17"/>
-      <c r="N32" s="44"/>
-      <c r="O32" s="44"/>
+      <c r="N32" s="17"/>
+      <c r="O32" s="17"/>
     </row>
     <row r="33" spans="2:15" ht="18.75" x14ac:dyDescent="0.25">
       <c r="B33" s="29" t="s">
@@ -2737,17 +2728,17 @@
         <v>6.01</v>
       </c>
       <c r="J33" s="17"/>
-      <c r="K33" s="47">
+      <c r="K33" s="43">
         <v>4.09</v>
       </c>
-      <c r="L33" s="43">
+      <c r="L33" s="42">
         <v>2.54</v>
       </c>
       <c r="M33" s="17"/>
-      <c r="N33" s="42">
+      <c r="N33" s="41">
         <v>1.61</v>
       </c>
-      <c r="O33" s="43">
+      <c r="O33" s="42">
         <v>-2.5</v>
       </c>
     </row>
@@ -2798,7 +2789,7 @@
       <c r="K36" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="N36" s="48"/>
+      <c r="N36" s="2"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -2806,6 +2797,6 @@
   </mergeCells>
   <phoneticPr fontId="6" type="noConversion"/>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" scale="67" orientation="landscape" r:id="rId1"/>
+  <pageSetup paperSize="8" scale="88" orientation="landscape" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>